<commit_message>
Publish chapter 4 workbooks and chapter 3 recap
</commit_message>
<xml_diff>
--- a/outputs/01a15558-33a2-7ab0-8172-87a04b40c77e/kapitel-04-beregninger.xlsx
+++ b/outputs/01a15558-33a2-7ab0-8172-87a04b40c77e/kapitel-04-beregninger.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.1" sheetId="1" r:id="R0e7fef2c0a564dfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.2" sheetId="2" r:id="Rc2e9eb3421ce4f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.3" sheetId="3" r:id="R3a0520b67f4841d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.4" sheetId="4" r:id="R59995f87705f400e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.5" sheetId="5" r:id="Rbe5067e6f9fb4b6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.6" sheetId="6" r:id="Re9d77af7aa3e49e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.7" sheetId="7" r:id="R079034469a1d4393"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.1" sheetId="1" r:id="Re74aafb8d7864334"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.2" sheetId="2" r:id="R8abd7f3435da454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.3" sheetId="3" r:id="R49851076a7644b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.4" sheetId="4" r:id="R387cbb3815844e56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.5" sheetId="5" r:id="Rfbd0feeb911843b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.6" sheetId="6" r:id="Rd934e529693249ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.7" sheetId="7" r:id="R09f93126e5a74878"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -366,7 +366,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Hvor ligger obligationernes værdi i tid?</a:t>
+              <a:t>Hvert års nutidsværdi som andel af kursen</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -394,7 +394,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>S: PV-vægt</c:v>
+            <c:v>S: andel af kursen</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -424,7 +424,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>A: PV-vægt</c:v>
+            <c:v>A: andel af kursen</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -587,7 +587,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Krumningen forklarer forskellen</a:t>
+              <a:t>Faktisk kurs og to estimater</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -911,7 +911,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Kursfald</c:v>
+            <c:v>Kursfald, kurspoint</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -1066,7 +1066,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re78da718ee4d454a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R846dd47a28bf46cc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1101,7 +1101,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdf1ae719f3504c6c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfec5e239f3a3453b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1136,7 +1136,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ea3fcc96f044be2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R024a4022abd84fa5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1680,7 +1680,7 @@
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="2"/>
       <x:c r="B20" s="26" t="str">
-        <x:v>Kurs / varighed i år</x:v>
+        <x:v>Kurs og Macaulay-varighed, år</x:v>
       </x:c>
       <x:c r="C20" s="26"/>
       <x:c r="D20" s="26"/>
@@ -1713,10 +1713,10 @@
         <x:v>År</x:v>
       </x:c>
       <x:c r="C22" s="18" t="str">
-        <x:v>S: PV-vægt</x:v>
+        <x:v>S: andel af kursen</x:v>
       </x:c>
       <x:c r="D22" s="18" t="str">
-        <x:v>A: PV-vægt</x:v>
+        <x:v>A: andel af kursen</x:v>
       </x:c>
       <x:c r="E22" s="2"/>
       <x:c r="F22" s="2"/>
@@ -1987,7 +1987,7 @@
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="2"/>
       <x:c r="B35" s="26" t="str">
-        <x:v>Kurs / varighed i år</x:v>
+        <x:v>Kurs og Macaulay-varighed, år</x:v>
       </x:c>
       <x:c r="C35" s="26"/>
       <x:c r="D35" s="26"/>
@@ -2067,7 +2067,7 @@
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="A41" s="2"/>
       <x:c r="B41" s="13" t="str">
-        <x:v>A flytter derfor mere værdi til tidligere år: tyngdepunktet ligger tidligere, og varigheden er kortere.</x:v>
+        <x:v>A's betalinger kommer tidligere, så en større del af kursen stammer fra de første år. Varigheden bliver kortere.</x:v>
       </x:c>
       <x:c r="C41" s="13"/>
       <x:c r="D41" s="13"/>
@@ -2104,7 +2104,7 @@
     <x:row r="44" ht="24" customHeight="1">
       <x:c r="A44" s="2"/>
       <x:c r="B44" s="13" t="str">
-        <x:v>3,68 år er en vægtet gennemsnitstid. Der kommer ingen betaling på netop det tidspunkt.</x:v>
+        <x:v>S's varighed i H20 er en vægtet gennemsnitstid. Der falder ingen betaling på netop det tidspunkt.</x:v>
       </x:c>
       <x:c r="C44" s="13"/>
       <x:c r="D44" s="13"/>
@@ -2360,7 +2360,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b98722dbba049cc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e34d55c902b49db"/>
 </x:worksheet>
 </file>
 
@@ -2538,7 +2538,7 @@
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="2"/>
       <x:c r="B13" s="2" t="str">
-        <x:v>Modificeret varighed</x:v>
+        <x:v>Modificeret varighed, %/pp</x:v>
       </x:c>
       <x:c r="C13" s="23" t="n">
         <x:f>C8/(1+C9)</x:f>
@@ -2610,7 +2610,7 @@
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="2"/>
       <x:c r="B18" s="13" t="str">
-        <x:v>pp = procentpoint; bp = basispunkt. Risikomålene vises positive; en rentestigning giver et kurstab.</x:v>
+        <x:v>pp = procentpoint; bp = basispunkt. Risikomålene vises som positive tal; en rentestigning giver et kurstab.</x:v>
       </x:c>
       <x:c r="C18" s="13"/>
       <x:c r="D18" s="13"/>
@@ -2721,7 +2721,7 @@
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="2"/>
       <x:c r="B26" s="2" t="str">
-        <x:v>Estimeret ændring, kurspoint</x:v>
+        <x:v>Estimeret kursændring, kurspoint</x:v>
       </x:c>
       <x:c r="C26" s="19" t="n">
         <x:f>-C14*C24</x:f>
@@ -2834,7 +2834,7 @@
     <x:row r="34" ht="24" customHeight="1">
       <x:c r="A34" s="2"/>
       <x:c r="B34" s="2" t="str">
-        <x:v>Estimeret kronetab</x:v>
+        <x:v>Estimeret tab, kr.</x:v>
       </x:c>
       <x:c r="C34" s="40" t="n">
         <x:f>C33*C13*C32/10000</x:f>
@@ -2861,7 +2861,7 @@
     <x:row r="36" ht="24" customHeight="1">
       <x:c r="A36" s="2"/>
       <x:c r="B36" s="13" t="str">
-        <x:v>Tabet er positivt her. Det er markedsværdien, der ganges med den procentvise kursnedgang.</x:v>
+        <x:v>Tabet vises som et positivt beløb. Det er markedsværdien, ikke det nominelle beløb, der ganges med den procentvise kursnedgang.</x:v>
       </x:c>
       <x:c r="C36" s="13"/>
       <x:c r="D36" s="13"/>
@@ -2911,7 +2911,7 @@
     <x:row r="40" ht="24" customHeight="1">
       <x:c r="A40" s="2"/>
       <x:c r="B40" s="13" t="str">
-        <x:v>MD × renteændring som decimal giver en relativ ændring. Gang derefter med kursen for at få kurspoint.</x:v>
+        <x:v>MD × renteændring som decimaltal giver den procentvise kursændring. Gang med kursen for at få kurspoint.</x:v>
       </x:c>
       <x:c r="C40" s="13"/>
       <x:c r="D40" s="13"/>
@@ -2959,7 +2959,7 @@
     <x:row r="44" ht="24" customHeight="1">
       <x:c r="A44" s="2"/>
       <x:c r="B44" s="13" t="str">
-        <x:v>Der regnes videre med uafrundede tal fra 4.1; små forskelle fra afrundede tal i slides kan forekomme.</x:v>
+        <x:v>Regnearket bruger uafrundede tal fra 4.1, så resultaterne kan afvige lidt fra afrundede facitter.</x:v>
       </x:c>
       <x:c r="C44" s="13"/>
       <x:c r="D44" s="13"/>
@@ -3171,7 +3171,7 @@
         <x:v>År × (år + 1)</x:v>
       </x:c>
       <x:c r="F13" s="18" t="str">
-        <x:v>Bidrag til summen</x:v>
+        <x:v>Nutidsværdi × år × (år + 1)</x:v>
       </x:c>
       <x:c r="G13" s="2"/>
       <x:c r="H13" s="2"/>
@@ -3334,7 +3334,7 @@
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="2"/>
       <x:c r="B22" s="13" t="str">
-        <x:v>Divider summen med (1 + rente)² og med 10.000. Så kan renteændringen indsættes i procentpoint.</x:v>
+        <x:v>Del summen med (1 + rente)² og med 10.000, så renteændringen kan indsættes i procentpoint.</x:v>
       </x:c>
       <x:c r="C22" s="13"/>
       <x:c r="D22" s="13"/>
@@ -3391,16 +3391,16 @@
         <x:v>Faktisk kurs</x:v>
       </x:c>
       <x:c r="E26" s="18" t="str">
-        <x:v>Faktisk ændring</x:v>
+        <x:v>Faktisk kursændring</x:v>
       </x:c>
       <x:c r="F26" s="18" t="str">
-        <x:v>Kun varighed</x:v>
+        <x:v>Estimat: kun varighed</x:v>
       </x:c>
       <x:c r="G26" s="18" t="str">
         <x:v>Konveksitetsled</x:v>
       </x:c>
       <x:c r="H26" s="18" t="str">
-        <x:v>Begge led</x:v>
+        <x:v>Estimat: med konveksitet</x:v>
       </x:c>
       <x:c r="I26" s="2"/>
     </x:row>
@@ -3517,7 +3517,7 @@
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="2"/>
       <x:c r="B33" s="13" t="str">
-        <x:v>Varighed alene undervurderer gevinsten ved rentefald og overvurderer tabet ved rentestigning.</x:v>
+        <x:v>S har positiv konveksitet. Derfor undervurderer varighed alene gevinsten ved rentefald og overvurderer tabet ved rentestigning.</x:v>
       </x:c>
       <x:c r="C33" s="13"/>
       <x:c r="D33" s="13"/>
@@ -3530,7 +3530,7 @@
     <x:row r="34" ht="24" customHeight="1">
       <x:c r="A34" s="2"/>
       <x:c r="B34" s="13" t="str">
-        <x:v>For denne obligation er konveksiteten positiv. Korrektionen er derfor positiv i begge retninger.</x:v>
+        <x:v>Konveksitetsleddet er positivt, uanset om renten stiger eller falder.</x:v>
       </x:c>
       <x:c r="C34" s="13"/>
       <x:c r="D34" s="13"/>
@@ -3543,7 +3543,7 @@
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="2"/>
       <x:c r="B35" s="13" t="str">
-        <x:v>Varighed plus konveksitet kommer tættere på. Den faktiske kurs kræver, at alle betalinger prises igen.</x:v>
+        <x:v>Varighed plus konveksitet kommer tættere på. Den faktiske kurs fås kun ved at diskontere alle betalinger med den nye rente.</x:v>
       </x:c>
       <x:c r="C35" s="13"/>
       <x:c r="D35" s="13"/>
@@ -4096,7 +4096,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8a71d8eaa734a0d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f78c968233f4ac6"/>
 </x:worksheet>
 </file>
 
@@ -4214,13 +4214,13 @@
         <x:v>Markedsværdi, kr.</x:v>
       </x:c>
       <x:c r="F8" s="18" t="str">
-        <x:v>Mod. varighed</x:v>
+        <x:v>Modificeret varighed</x:v>
       </x:c>
       <x:c r="G8" s="18" t="str">
-        <x:v>MV-vægt</x:v>
+        <x:v>Vægt efter markedsværdi</x:v>
       </x:c>
       <x:c r="H8" s="18" t="str">
-        <x:v>Kronevarighed</x:v>
+        <x:v>Kronevarighed, kurspoint/pp</x:v>
       </x:c>
       <x:c r="I8" s="2"/>
     </x:row>
@@ -4343,7 +4343,7 @@
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="2"/>
       <x:c r="B15" s="2" t="str">
-        <x:v>Juniorens nominelle vægtning</x:v>
+        <x:v>Juniorens varighed (nominelle vægte)</x:v>
       </x:c>
       <x:c r="C15" s="19" t="n">
         <x:f>SUMPRODUCT(C9:C10,F9:F10)/C11</x:f>
@@ -4397,7 +4397,7 @@
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="2"/>
       <x:c r="B19" s="13" t="str">
-        <x:v>Modificeret varighed vægtes med markedsværdier: 32/44 og 12/44.</x:v>
+        <x:v>Modificeret varighed vægtes med markedsværdier, fordi den måler den procentvise ændring i markedsværdien.</x:v>
       </x:c>
       <x:c r="C19" s="13"/>
       <x:c r="D19" s="13"/>
@@ -4410,7 +4410,7 @@
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="2"/>
       <x:c r="B20" s="13" t="str">
-        <x:v>Kronevarighed pr. 100 nominel vægtes med nominelle beløb: 40/50 og 10/50.</x:v>
+        <x:v>Kronevarighed pr. 100 nominel vægtes med nominelle beløb, fordi kursen allerede indgår i den.</x:v>
       </x:c>
       <x:c r="C20" s="13"/>
       <x:c r="D20" s="13"/>
@@ -4473,7 +4473,7 @@
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="2"/>
       <x:c r="B25" s="2" t="str">
-        <x:v>Tab via modificeret varighed</x:v>
+        <x:v>Tab via modificeret varighed, kr.</x:v>
       </x:c>
       <x:c r="C25" s="40" t="n">
         <x:f>E11*C14*C24/100</x:f>
@@ -4489,7 +4489,7 @@
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="2"/>
       <x:c r="B26" s="2" t="str">
-        <x:v>Tab via kronevarighed</x:v>
+        <x:v>Tab via kronevarighed, kr.</x:v>
       </x:c>
       <x:c r="C26" s="40" t="n">
         <x:f>C11/100*C17*C24</x:f>
@@ -4588,7 +4588,7 @@
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="2"/>
       <x:c r="B33" s="2" t="str">
-        <x:v>MD × porteføljekurs / 100</x:v>
+        <x:v>Modificeret varighed × kurs / 100</x:v>
       </x:c>
       <x:c r="C33" s="19" t="n">
         <x:f>C14*C32/100</x:f>
@@ -4620,7 +4620,7 @@
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="2"/>
       <x:c r="B35" s="2" t="str">
-        <x:v>Undervurderet tab, kr.</x:v>
+        <x:v>Juniorens undervurdering, kr.</x:v>
       </x:c>
       <x:c r="C35" s="40" t="n">
         <x:f>C25-C34</x:f>
@@ -4647,7 +4647,7 @@
     <x:row r="37" ht="24" customHeight="1">
       <x:c r="A37" s="2"/>
       <x:c r="B37" s="13" t="str">
-        <x:v>Obligation 2 har høj varighed og kurs 120. Den fylder mere i markedsværdi end i nominelt beløb.</x:v>
+        <x:v>Med opgavens tal har obligation 2 både den højeste varighed og en kurs over 100. Den vejer derfor mere i markedsværdi end nominelt.</x:v>
       </x:c>
       <x:c r="C37" s="13"/>
       <x:c r="D37" s="13"/>
@@ -4674,10 +4674,10 @@
         <x:v>Obligation</x:v>
       </x:c>
       <x:c r="C39" s="18" t="str">
-        <x:v>Nominel vægt</x:v>
+        <x:v>Vægt efter nominel værdi</x:v>
       </x:c>
       <x:c r="D39" s="18" t="str">
-        <x:v>Markedsværdivægt</x:v>
+        <x:v>Vægt efter markedsværdi</x:v>
       </x:c>
       <x:c r="E39" s="2"/>
       <x:c r="F39" s="2"/>
@@ -4737,7 +4737,7 @@
     <x:row r="43" ht="24" customHeight="1">
       <x:c r="A43" s="2"/>
       <x:c r="B43" s="13" t="str">
-        <x:v>Nominelle vægte: 80 % og 20 %. Markedsværdivægte: ca. 72,73 % og 27,27 %.</x:v>
+        <x:v>Junioren giver den mest rentefølsomme obligation for lille vægt og undervurderer derfor risikoen.</x:v>
       </x:c>
       <x:c r="C43" s="13"/>
       <x:c r="D43" s="13"/>
@@ -4749,15 +4749,13 @@
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
       <x:c r="A44" s="2"/>
-      <x:c r="B44" s="13" t="str">
-        <x:v>Junioren giver den mest rentefølsomme obligation for lille vægt og undervurderer derfor risikoen.</x:v>
-      </x:c>
-      <x:c r="C44" s="13"/>
-      <x:c r="D44" s="13"/>
-      <x:c r="E44" s="13"/>
-      <x:c r="F44" s="13"/>
-      <x:c r="G44" s="13"/>
-      <x:c r="H44" s="13"/>
+      <x:c r="B44" s="2"/>
+      <x:c r="C44" s="2"/>
+      <x:c r="D44" s="2"/>
+      <x:c r="E44" s="2"/>
+      <x:c r="F44" s="2"/>
+      <x:c r="G44" s="2"/>
+      <x:c r="H44" s="2"/>
       <x:c r="I44" s="2"/>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
@@ -4924,7 +4922,7 @@
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="2"/>
       <x:c r="B8" s="2" t="str">
-        <x:v>Betaling om 7 år, kr.</x:v>
+        <x:v>Forpligtelse, kr.</x:v>
       </x:c>
       <x:c r="C8" s="38" t="n">
         <x:v>10000000</x:v>
@@ -4980,7 +4978,7 @@
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="2"/>
       <x:c r="B12" s="2" t="str">
-        <x:v>Beløb, der skal afsættes i dag</x:v>
+        <x:v>Nutidsværdi af forpligtelsen, kr.</x:v>
       </x:c>
       <x:c r="C12" s="40" t="n">
         <x:f>C8/(1+C10)^C9</x:f>
@@ -5034,13 +5032,13 @@
         <x:v>Obligation</x:v>
       </x:c>
       <x:c r="C16" s="18" t="str">
-        <x:v>Macaulay, år</x:v>
+        <x:v>Varighed, år</x:v>
       </x:c>
       <x:c r="D16" s="18" t="str">
-        <x:v>Horisont minus D</x:v>
+        <x:v>Horisont minus varighed, år</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
-        <x:v>Valg ved opgavens input</x:v>
+        <x:v>Varighed i forhold til horisont</x:v>
       </x:c>
       <x:c r="F16" s="2"/>
       <x:c r="G16" s="2"/>
@@ -5124,7 +5122,7 @@
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="2"/>
       <x:c r="B21" s="13" t="str">
-        <x:v>Forpligtelsen er én betaling om 7 år: dens Macaulay-varighed er 7 år. Y har samme varighed.</x:v>
+        <x:v>Forpligtelsen er én betaling på horisonten, så dens Macaulay-varighed er lig horisonten.</x:v>
       </x:c>
       <x:c r="C21" s="13"/>
       <x:c r="D21" s="13"/>
@@ -5137,7 +5135,7 @@
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="2"/>
       <x:c r="B22" s="13" t="str">
-        <x:v>Invester forpligtelsens nutidsværdi i Y. Dermed matches værdi og førsteordensfølsomhed i dag.</x:v>
+        <x:v>Investér nutidsværdien i Y. Så har aktiv og forpligtelse samme værdi og reagerer ens på en lille parallel renteændring.</x:v>
       </x:c>
       <x:c r="C22" s="13"/>
       <x:c r="D22" s="13"/>
@@ -5185,7 +5183,7 @@
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="2"/>
       <x:c r="B26" s="13" t="str">
-        <x:v>X ved rentefald: tidlige betalinger skal genplaceres til lavere renter frem mod år 7.</x:v>
+        <x:v>X ved rentefald: X's betalinger modtages før horisonten og må geninvesteres til den lavere rente.</x:v>
       </x:c>
       <x:c r="C26" s="13"/>
       <x:c r="D26" s="13"/>
@@ -5198,7 +5196,7 @@
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="2"/>
       <x:c r="B27" s="13" t="str">
-        <x:v>Kursgevinsten opvejer ikke hele tabet af genplaceringsafkast. Slutværdien falder i første orden.</x:v>
+        <x:v>Kursgevinsten opvejer ikke det lavere afkast på de geninvesterede betalinger, så værdien på horisonten bliver mindre end forpligtelsen.</x:v>
       </x:c>
       <x:c r="C27" s="13"/>
       <x:c r="D27" s="13"/>
@@ -5222,7 +5220,7 @@
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="2"/>
       <x:c r="B29" s="13" t="str">
-        <x:v>Z ved rentestigning: kursfaldet dominerer gevinsten fra højere genplaceringsrente frem mod år 7.</x:v>
+        <x:v>Z ved rentestigning: Z's betalinger efter horisonten skal sælges, og deres salgsværdi falder.</x:v>
       </x:c>
       <x:c r="C29" s="13"/>
       <x:c r="D29" s="13"/>
@@ -5235,7 +5233,7 @@
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="2"/>
       <x:c r="B30" s="13" t="str">
-        <x:v>Betalinger efter år 7 indgår i salgsværdien på horisonten. Den værdi falder, når renten stiger.</x:v>
+        <x:v>Faldet er større end gevinsten ved at geninvestere de tidlige betalinger til den højere rente.</x:v>
       </x:c>
       <x:c r="C30" s="13"/>
       <x:c r="D30" s="13"/>
@@ -5259,7 +5257,7 @@
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="2"/>
       <x:c r="B32" s="6" t="str">
-        <x:v>(c) Horisonten gennem betalingernes tyngdepunkt</x:v>
+        <x:v>(c) Når horisonten svarer til varigheden</x:v>
       </x:c>
       <x:c r="C32" s="6"/>
       <x:c r="D32" s="6"/>
@@ -5283,7 +5281,7 @@
     <x:row r="34" ht="24" customHeight="1">
       <x:c r="A34" s="2"/>
       <x:c r="B34" s="13" t="str">
-        <x:v>Tidlige betalinger genplaceres frem til horisonten; senere betalinger indgår via salgsværdien dér.</x:v>
+        <x:v>Betalinger før horisonten geninvesteres frem til horisonten. Betalinger efter horisonten sælges dér til markedskurs.</x:v>
       </x:c>
       <x:c r="C34" s="13"/>
       <x:c r="D34" s="13"/>
@@ -5296,7 +5294,7 @@
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="2"/>
       <x:c r="B35" s="13" t="str">
-        <x:v>Ved H = D balancerer de to rentevirkninger for et lille, varigt parallelt renteskift.</x:v>
+        <x:v>Når horisonten er lig varigheden, opvejer de to virkninger hinanden ved et lille parallelt renteskift lige efter købet.</x:v>
       </x:c>
       <x:c r="C35" s="13"/>
       <x:c r="D35" s="13"/>
@@ -5309,7 +5307,7 @@
     <x:row r="36" ht="24" customHeight="1">
       <x:c r="A36" s="2"/>
       <x:c r="B36" s="13" t="str">
-        <x:v>Y har derfor ingen førsteordensændring i slutværdien. Det er ikke en garanti mod alle rentebevægelser.</x:v>
+        <x:v>Værdien på horisonten ændres så kun lidt. Store skift, ændret kurveform eller flere skift undervejs kan stadig give afvigelser.</x:v>
       </x:c>
       <x:c r="C36" s="13"/>
       <x:c r="D36" s="13"/>
@@ -5357,7 +5355,7 @@
     <x:row r="40" ht="24" customHeight="1">
       <x:c r="A40" s="2"/>
       <x:c r="B40" s="13" t="str">
-        <x:v>1. Tiden går og kuponer betales. Obligationens varighed falder ikke nødvendigvis i takt med horisonten.</x:v>
+        <x:v>1. Når tiden går, falder horisonten ét år pr. år, men obligationens varighed falder ikke nødvendigvis lige så hurtigt.</x:v>
       </x:c>
       <x:c r="C40" s="13"/>
       <x:c r="D40" s="13"/>
@@ -5370,7 +5368,7 @@
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="A41" s="2"/>
       <x:c r="B41" s="13" t="str">
-        <x:v>2. Renter ændrer nutidsværdierne og dermed varigheden. Værdi- og varighedsmatch skal kontrolleres igen.</x:v>
+        <x:v>2. Når renten ændrer sig, ændres nutidsværdierne og dermed varigheden. Matchet skal derfor kontrolleres igen.</x:v>
       </x:c>
       <x:c r="C41" s="13"/>
       <x:c r="D41" s="13"/>
@@ -5394,7 +5392,7 @@
     <x:row r="43" ht="24" customHeight="1">
       <x:c r="A43" s="2"/>
       <x:c r="B43" s="13" t="str">
-        <x:v>Forudsætning: små parallelle renteskift i den enkle model med fast betalingsrække og fælles rente.</x:v>
+        <x:v>Forudsætninger: samme rente for alle løbetider, små parallelle renteskift og faste, kendte betalinger.</x:v>
       </x:c>
       <x:c r="C43" s="13"/>
       <x:c r="D43" s="13"/>
@@ -5611,7 +5609,7 @@
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="2"/>
       <x:c r="B9" s="2" t="str">
-        <x:v>Lokalt / parallelt stød, pp</x:v>
+        <x:v>Rentestød, procentpoint</x:v>
       </x:c>
       <x:c r="C9" s="9" t="n">
         <x:v>1</x:v>
@@ -5673,7 +5671,7 @@
         <x:v>Nutidsværdi</x:v>
       </x:c>
       <x:c r="F13" s="18" t="str">
-        <x:v>PV-vægt</x:v>
+        <x:v>Andel af kursen</x:v>
       </x:c>
       <x:c r="G13" s="18" t="str">
         <x:v>Vægt × år</x:v>
@@ -5765,7 +5763,7 @@
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="2"/>
       <x:c r="B17" s="26" t="str">
-        <x:v>Kurs / Fisher–Weil, år</x:v>
+        <x:v>Kurs og Fisher–Weil-varighed, år</x:v>
       </x:c>
       <x:c r="C17" s="26"/>
       <x:c r="D17" s="26"/>
@@ -5795,7 +5793,7 @@
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="2"/>
       <x:c r="B19" s="13" t="str">
-        <x:v>Fisher–Weil er her den PV-vægtede tid på spotkurven, som defineret i kapitlet.</x:v>
+        <x:v>Fisher–Weil-varighed er den gennemsnitlige betalingstid, vægtet med nutidsværdier beregnet på spotkurven.</x:v>
       </x:c>
       <x:c r="C19" s="13"/>
       <x:c r="D19" s="13"/>
@@ -5832,7 +5830,7 @@
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="2"/>
       <x:c r="B22" s="13" t="str">
-        <x:v>1 %, 2 % og 3 % priser hver sin betalingsdato. Bruges én af dem til alt, ændres kursen og vægtene.</x:v>
+        <x:v>Hver spotrente gælder én betalingsdato. Diskonteres alle betalinger med én af dem, ændres både kursen og vægtene.</x:v>
       </x:c>
       <x:c r="C22" s="13"/>
       <x:c r="D22" s="13"/>
@@ -5845,7 +5843,7 @@
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="2"/>
       <x:c r="B23" s="13" t="str">
-        <x:v>En effektiv rente kan findes, så samme kurs opnås, men den er ikke vilkårligt én af spotrenterne.</x:v>
+        <x:v>Én effektiv rente kan give samme kurs, men den skal beregnes. Den er ikke bare en af spotrenterne.</x:v>
       </x:c>
       <x:c r="C23" s="13"/>
       <x:c r="D23" s="13"/>
@@ -5899,19 +5897,19 @@
         <x:v>Ny spotrente</x:v>
       </x:c>
       <x:c r="D27" s="18" t="str">
-        <x:v>Gammel PV</x:v>
+        <x:v>Nutidsværdi før</x:v>
       </x:c>
       <x:c r="E27" s="18" t="str">
-        <x:v>Ny PV</x:v>
+        <x:v>Nutidsværdi efter</x:v>
       </x:c>
       <x:c r="F27" s="18" t="str">
-        <x:v>Kursfald</x:v>
+        <x:v>Kursfald, kurspoint</x:v>
       </x:c>
       <x:c r="G27" s="18" t="str">
         <x:v>Ny samlet kurs</x:v>
       </x:c>
       <x:c r="H27" s="18" t="str">
-        <x:v>Andel af fald</x:v>
+        <x:v>Andel af samlet fald</x:v>
       </x:c>
       <x:c r="I27" s="2"/>
     </x:row>
@@ -6100,7 +6098,7 @@
     <x:row r="37" ht="24" customHeight="1">
       <x:c r="A37" s="2"/>
       <x:c r="B37" s="13" t="str">
-        <x:v>Her rammer hvert lokalt stød præcis én separat betaling. Derfor gælder ligheden eksakt før afrunding.</x:v>
+        <x:v>Hvert lokalt stød rammer kun én betaling. Derfor er summen præcis lig kursfaldet ved det parallelle skift.</x:v>
       </x:c>
       <x:c r="C37" s="13"/>
       <x:c r="D37" s="13"/>
@@ -6113,7 +6111,7 @@
     <x:row r="38" ht="24" customHeight="1">
       <x:c r="A38" s="2"/>
       <x:c r="B38" s="13" t="str">
-        <x:v>Ved overlappende lokale stød gælder additivitet generelt kun som førsteordensapproksimation.</x:v>
+        <x:v>Rammer flere stød den samme betaling, er summen kun en tilnærmelse.</x:v>
       </x:c>
       <x:c r="C38" s="13"/>
       <x:c r="D38" s="13"/>
@@ -6292,7 +6290,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8abcc49853724064"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56d6573d4c50495f"/>
 </x:worksheet>
 </file>
 
@@ -6483,7 +6481,7 @@
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="2"/>
       <x:c r="B15" s="13" t="str">
-        <x:v>Opgave 4.3 viser forskellen: ved større stød hjælper konveksitet, mens genprisning giver den faktiske kurs.</x:v>
+        <x:v>Opgave 4.3 viser det: konveksitet bringer estimatet tættere på, men kun en ny prisberegning giver den faktiske kurs.</x:v>
       </x:c>
       <x:c r="C15" s="13"/>
       <x:c r="D15" s="13"/>
@@ -6542,7 +6540,7 @@
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="2"/>
       <x:c r="B20" s="13" t="str">
-        <x:v>Ved samme varighed forbedrer positiv konveksitet prisreaktionen i begge retninger.</x:v>
+        <x:v>Ved samme varighed giver højere konveksitet større kursgevinst ved rentefald og mindre kurstab ved rentestigning.</x:v>
       </x:c>
       <x:c r="C20" s="13"/>
       <x:c r="D20" s="13"/>
@@ -6555,7 +6553,7 @@
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="2"/>
       <x:c r="B21" s="13" t="str">
-        <x:v>Men fordelen kan være indregnet i en højere købspris og et lavere afkast. Højest konveksitet er ikke altid bedst.</x:v>
+        <x:v>Fordelen er typisk betalt via en højere kurs og dermed lavere effektiv rente. Mest konveksitet er ikke altid bedst.</x:v>
       </x:c>
       <x:c r="C21" s="13"/>
       <x:c r="D21" s="13"/>
@@ -6614,7 +6612,7 @@
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="2"/>
       <x:c r="B26" s="13" t="str">
-        <x:v>Nul samlet kronevarighed fjerner kun førsteordensfølsomheden over for det valgte parallelle rentestød.</x:v>
+        <x:v>Nul kronevarighed betyder kun, at et lille parallelt renteskift ikke ændrer værdien i det lineære estimat.</x:v>
       </x:c>
       <x:c r="C26" s="13"/>
       <x:c r="D26" s="13"/>
@@ -6627,7 +6625,7 @@
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="2"/>
       <x:c r="B27" s="13" t="str">
-        <x:v>Risiko ved ændret kurveform og konveksitet kan stadig være til stede. Se også de lokale stød i 4.6.</x:v>
+        <x:v>Ændret kurveform og store renteskift kan stadig give tab eller gevinst. Se de lokale stød i 4.6.</x:v>
       </x:c>
       <x:c r="C27" s="13"/>
       <x:c r="D27" s="13"/>

</xml_diff>